<commit_message>
Rename the incurred-cost example to a generic indirect-rates example
Same coverage (grouped pools, cross-sheet rates, named formulas, shared
formulas, protected sheet); neutral wording in the workbook, docs and tests.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/corpus/known-bad/j-orphan-shared-formula.xlsx
+++ b/corpus/known-bad/j-orphan-shared-formula.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\foxtr\LocalTools\excel-graft\corpus\templates\incurred-cost\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\foxtr\LocalTools\excel-graft\corpus\templates\indirect-rates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3C9A1567-4737-493C-AA01-64D344522111}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{70390287-EDB7-411A-9C46-50885EBD4CEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2240" yWindow="2470" windowWidth="28800" windowHeight="15910" xr2:uid="{C05344DF-DDB8-4915-9AF2-BF8468360296}"/>
+    <workbookView xWindow="2240" yWindow="2470" windowWidth="28800" windowHeight="15910" xr2:uid="{35E72F41-FF67-41FF-A7A4-5570E7BDCA79}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -55,10 +55,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="58">
   <si>
-    <t>Incurred Cost Electronic Submission</t>
-  </si>
-  <si>
-    <t>Prepared in accordance with FAR 52.216-7(d)(2) - Schedules H, H-1 and supporting pools</t>
+    <t>Indirect Cost Rates</t>
+  </si>
+  <si>
+    <t>Annual indirect cost pools, allocation bases and rates</t>
   </si>
   <si>
     <t>Contractor</t>
@@ -641,7 +641,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-E148-4F2F-927F-EC8D77E3B4DF}"/>
+              <c16:uniqueId val="{00000000-F2CB-4393-B41E-6716C1329B10}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -706,7 +706,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-E148-4F2F-927F-EC8D77E3B4DF}"/>
+              <c16:uniqueId val="{00000001-F2CB-4393-B41E-6716C1329B10}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -719,11 +719,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="182"/>
-        <c:axId val="774301664"/>
-        <c:axId val="1451544623"/>
+        <c:axId val="285190032"/>
+        <c:axId val="277363888"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="774301664"/>
+        <c:axId val="285190032"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -766,7 +766,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1451544623"/>
+        <c:crossAx val="277363888"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -774,7 +774,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1451544623"/>
+        <c:axId val="277363888"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -825,7 +825,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="774301664"/>
+        <c:crossAx val="285190032"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1446,7 +1446,7 @@
         <xdr:cNvPr id="2" name="RatesChart">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{35855EB1-E5F1-0918-253D-4A0CD8BE20BE}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{99947945-9935-0A60-F092-63E68CDEDD0C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1468,15 +1468,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{817FF9EB-CECB-483A-8748-78303EF1213B}" name="DirectLabor" displayName="DirectLabor" ref="A4:F11" totalsRowCount="1">
-  <autoFilter ref="A4:F10" xr:uid="{817FF9EB-CECB-483A-8748-78303EF1213B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FCBA1F05-7631-4F7D-B156-ED93FB144A9A}" name="DirectLabor" displayName="DirectLabor" ref="A4:F11" totalsRowCount="1">
+  <autoFilter ref="A4:F10" xr:uid="{FCBA1F05-7631-4F7D-B156-ED93FB144A9A}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{1FA67AE5-7126-4647-AA6D-CD4C29137287}" name="Employee" totalsRowLabel="Total"/>
-    <tableColumn id="2" xr3:uid="{84CCCAD7-4975-4CE5-876C-D6BA941F11C3}" name="LaborCategory"/>
-    <tableColumn id="3" xr3:uid="{1CF75557-1517-4BBF-BF77-D96CB0B8D58E}" name="Project"/>
-    <tableColumn id="4" xr3:uid="{191CDE0A-953A-4C98-A294-20E0604F030B}" name="Hours" totalsRowFunction="sum" dataDxfId="4" totalsRowDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{93531859-296A-4E4D-8FDA-8E4026BBB71C}" name="Rate" dataDxfId="2" totalsRowDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{A292CCA6-CDA5-46ED-9093-EF2A333F76F3}" name="Cost" totalsRowFunction="sum" dataDxfId="1" totalsRowDxfId="0">
+    <tableColumn id="1" xr3:uid="{81FF66AD-2AAF-4F10-84D6-47FE9635F33C}" name="Employee" totalsRowLabel="Total"/>
+    <tableColumn id="2" xr3:uid="{155AD87C-D2C7-4F43-B248-26768DCEB99B}" name="LaborCategory"/>
+    <tableColumn id="3" xr3:uid="{550A8781-21DE-456D-AD2F-0FDAD260ACB6}" name="Project"/>
+    <tableColumn id="4" xr3:uid="{B85BA46F-BEAF-47CD-ADD1-2523C55D64A1}" name="Hours" totalsRowFunction="sum" dataDxfId="4" totalsRowDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{83542A76-DE6C-4395-95B3-E8130A5F59B1}" name="Rate" dataDxfId="2" totalsRowDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{3B6FE450-1FBD-422D-AC29-A43CB7BFBF7D}" name="Cost" totalsRowFunction="sum" dataDxfId="1" totalsRowDxfId="0">
       <calculatedColumnFormula>DirectLabor[[#This Row],[Hours]]*DirectLabor[[#This Row],[Rate]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1746,7 +1746,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17DCED1B-8DE3-4E1C-96B9-20DA4911DAAB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51B881D4-E26D-4E9E-BD31-64E00CEC7CB7}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1819,7 +1819,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39F7E6D8-6A80-43B5-9856-F8AB2D77BF88}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF8EBDBB-0F6E-4C3D-A9B6-F217A1DB907E}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2018,7 +2018,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B013D65-1E32-447E-8FF5-74EFEF4D4D92}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20D1D671-CEA3-470D-8524-4468ED831CB9}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2257,7 +2257,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1B70204-F89C-40E1-B948-32C90D920D02}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14DD62CC-261C-4997-917C-769C9D536788}">
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>